<commit_message>
Sauvegarde complète du repo + correction Synthèse F&B
Inclut tous les chantiers en cours (gouvernance, mécénat, officiel,
programmation, organisation, scripts, subventions, communication, devis,
A_FAIRE) + correction des références Synthèse vers les nouvelles lignes
F&B (D16 recettes / D57 coûts).

.gitignore mis à jour pour exclure .claude/ (qui contient des secrets
OAuth Google détectés par GitHub push protection).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/budget/Suivi_budgetaire_Monique_Festival.xlsx
+++ b/budget/Suivi_budgetaire_Monique_Festival.xlsx
@@ -825,11 +825,11 @@
         </is>
       </c>
       <c r="B6" s="3">
-        <f>'F&amp;B'!D13</f>
+        <f>'F&amp;B'!D16</f>
         <v/>
       </c>
       <c r="C6" s="3">
-        <f>'F&amp;B'!E13</f>
+        <f>'F&amp;B'!E16</f>
         <v/>
       </c>
       <c r="D6" s="3">
@@ -837,11 +837,11 @@
         <v/>
       </c>
       <c r="E6" s="4">
-        <f>'F&amp;B'!D27</f>
+        <f>'F&amp;B'!D57</f>
         <v/>
       </c>
       <c r="F6" s="4">
-        <f>'F&amp;B'!E27</f>
+        <f>'F&amp;B'!E57</f>
         <v/>
       </c>
       <c r="G6" s="4">

</xml_diff>

<commit_message>
Synthèse : MAJ scénarios par jauge avec hypothèses F&B Scénario B
Mise à jour des scénarios de marge globale du festival pour refléter
les nouvelles hypothèses F&B :
- Δ Recettes vs initial : -1 061 € (31 381 € vs 32 442 €)
- Δ Coûts vs initial : +1 900 € (9 825 € vs 7 925 €)
- Δ Marge vs initial : -2 961 €

Nouveaux scénarios :
- Jauge -20% (960 fest) : Marge -3 264 €
- Jauge standard (1 200 fest) : Marge 5 614 €
- Jauge +20% (1 440 fest) : Marge 14 491 €
- Standard + réassort bière 5 fûts (+2 800 € marge) : 8 414 €

Note : SACEM 1 427 € et repas artistes 555 € exclus du F&B
(à imputer Droits d'auteur / Artistes si confirmés dus).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/budget/Suivi_budgetaire_Monique_Festival.xlsx
+++ b/budget/Suivi_budgetaire_Monique_Festival.xlsx
@@ -26,7 +26,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0\ \€"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -100,6 +100,15 @@
     </font>
     <font>
       <i val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="001F4E78"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00666666"/>
       <sz val="9"/>
     </font>
   </fonts>
@@ -240,7 +249,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -299,6 +308,8 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -664,7 +675,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="35" customWidth="1" style="18" min="1" max="1"/>
@@ -1095,13 +1106,13 @@
         </is>
       </c>
       <c r="B18" s="9" t="n">
-        <v>47464</v>
+        <v>46403</v>
       </c>
       <c r="C18" s="9" t="n">
-        <v>47767</v>
+        <v>49667</v>
       </c>
       <c r="D18" s="10" t="n">
-        <v>-303</v>
+        <v>-3264</v>
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
@@ -1119,13 +1130,13 @@
         </is>
       </c>
       <c r="B19" s="12" t="n">
-        <v>58482</v>
+        <v>57421</v>
       </c>
       <c r="C19" s="12" t="n">
-        <v>49907</v>
+        <v>51807</v>
       </c>
       <c r="D19" s="13" t="n">
-        <v>8575</v>
+        <v>5614</v>
       </c>
       <c r="E19" s="11" t="inlineStr">
         <is>
@@ -1143,13 +1154,13 @@
         </is>
       </c>
       <c r="B20" s="9" t="n">
-        <v>69500</v>
+        <v>68439</v>
       </c>
       <c r="C20" s="9" t="n">
-        <v>52048</v>
+        <v>53948</v>
       </c>
       <c r="D20" s="14" t="n">
-        <v>17453</v>
+        <v>14491</v>
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
@@ -1158,6 +1169,37 @@
       </c>
       <c r="F20" s="8" t="n">
         <v>1440</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="38" t="inlineStr">
+        <is>
+          <t>Standard + réassort bière 5 fûts</t>
+        </is>
+      </c>
+      <c r="B22" s="38" t="n">
+        <v>60621</v>
+      </c>
+      <c r="C22" s="38" t="n">
+        <v>52207</v>
+      </c>
+      <c r="D22" s="38" t="n">
+        <v>8414</v>
+      </c>
+      <c r="E22" s="38" t="inlineStr">
+        <is>
+          <t>1 200</t>
+        </is>
+      </c>
+      <c r="F22" s="38" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="39" t="inlineStr">
+        <is>
+          <t>Note : SACEM 1 427 € et repas artistes 555 € exclus du F&amp;B (à imputer Droits d auteur / Artistes si confirmes dus)</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>